<commit_message>
Fix: Remove duplicate App.js, correct API endpoint
</commit_message>
<xml_diff>
--- a/backend/data/owners.xlsx
+++ b/backend/data/owners.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H3"/>
   <cols>
     <col min="1" max="1" width="15.83203125" customWidth="1"/>
     <col min="2" max="2" width="15.83203125" customWidth="1"/>
@@ -461,9 +461,35 @@
         <v>6/9/2026, 2:47:20 am</v>
       </c>
     </row>
+    <row r="3">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Independent House</v>
+      </c>
+      <c r="C3" t="str">
+        <v>TEST-001</v>
+      </c>
+      <c r="D3" t="str">
+        <v>-</v>
+      </c>
+      <c r="E3" t="str">
+        <v>-</v>
+      </c>
+      <c r="F3" t="str">
+        <v>Test User</v>
+      </c>
+      <c r="G3" t="str">
+        <v>9876543210</v>
+      </c>
+      <c r="H3" t="str">
+        <v>6/9/2026, 12:18:35 pm</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H3"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>